<commit_message>
Pipeline: fill in contract values for the three TES teaming opps
Update the placeholder $0 estimates added earlier for the TES joint-pursuit
opportunities, sourced from the TES capture workbook (comparable-award
analysis, value-point estimates):

- OPP-006 CBO SENTRY (CB26-RFQ0012)      $0 -> $30,000,000
- OPP-007 CDC IFMS    (75D301-26-Q-78924) $0 ->  $4,500,000
- OPP-008 VA          (36C10B26Q0107)     $0 -> $20,000,000

Notes refreshed with the estimate basis/range, confidence, and capture
verdict (SENTRY=CONDITIONAL, CDC IFMS=NO-BID, VA=PURSUE). Flagged that
solicitation 36C10B26Q0107 is VA VIPPS (Phase II), not "TERPS" as the row
title still reads - left for the operator to rename.

Open-pipeline total (Dashboard!D12) refreshed 14.5M -> 69.0M. Edited
surgically at the XML layer to preserve all 252 formula caches (LibreOffice
recalc is unavailable in this environment). verify_parse.js: 11/11 metrics
pass, 0 drift; 252 formulas, 0 errors.
</commit_message>
<xml_diff>
--- a/VBX_Command_Center_v1.xlsx
+++ b/VBX_Command_Center_v1.xlsx
@@ -2414,7 +2414,7 @@
       </c>
       <c r="D12" s="8" t="n">
         <f aca="false">SUMIFS(Pipeline!F5:F1000,Pipeline!E5:E1000,"&lt;&gt;Awarded",Pipeline!E5:E1000,"&lt;&gt;Lost",Pipeline!E5:E1000,"&lt;&gt;")</f>
-        <v>14500000</v>
+        <v>69000000</v>
       </c>
       <c r="E12" s="11" t="n">
         <f aca="false">COUNTIFS(Active_Projects!H:H,"Active")</f>
@@ -18329,7 +18329,7 @@
         </is>
       </c>
       <c r="F10" s="43" t="n">
-        <v>0</v>
+        <v>30000000</v>
       </c>
       <c r="G10" s="41" t="n">
         <v>46175</v>
@@ -18344,7 +18344,7 @@
       </c>
       <c r="J10" s="42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Teaming with The Enterprise Solutions (TES). Network/DevSecOps/Service Desk/Web Security/Cybersecurity DoWs (J2,J3,J6-J9). 12-mo base + 4 option yrs. Value TBD.</t>
+          <t xml:space="preserve">Teaming with The Enterprise Solutions (TES). Network/DevSecOps/Service Desk/Web Security/Cybersecurity DoWs (J2,J3,J6-J9). 12-mo base + 4 option yrs. Est. $30M point (range $20-50M BPA ceiling; comparable-award basis, Medium-Low confidence). Capture verdict: CONDITIONAL.</t>
         </is>
       </c>
     </row>
@@ -18375,7 +18375,7 @@
         </is>
       </c>
       <c r="F11" s="43" t="n">
-        <v>0</v>
+        <v>4500000</v>
       </c>
       <c r="G11" s="41" t="n">
         <v>46175</v>
@@ -18390,7 +18390,7 @@
       </c>
       <c r="J11" s="42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Teaming with The Enterprise Solutions (TES). NAICS 541512, GSA SIN 54151S, 100% small business set-aside. Base + 4 option yrs (PoP 7/1/2026). Value TBD.</t>
+          <t xml:space="preserve">Teaming with The Enterprise Solutions (TES). NAICS 541512, GSA SIN 54151S, 100% small business set-aside. Base + 4 option yrs (PoP 7/1/2026). Est. $4.5M point (range $3-6M; TRIRIGA comparable basis, Medium confidence). Capture verdict: NO-BID (COTS/reseller policy).</t>
         </is>
       </c>
     </row>
@@ -18421,7 +18421,7 @@
         </is>
       </c>
       <c r="F12" s="43" t="n">
-        <v>0</v>
+        <v>20000000</v>
       </c>
       <c r="G12" s="41" t="n">
         <v>46175</v>
@@ -18436,7 +18436,7 @@
       </c>
       <c r="J12" s="42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Teaming with The Enterprise Solutions (TES). TERPS PWS. NOTE: uploaded PDF body mislabeled vs filename - verify PWS scope. NAICS/value TBD.</t>
+          <t xml:space="preserve">Teaming with The Enterprise Solutions (TES). Sol. 36C10B26Q0107 = VA VIPPS (Phase II) per capture analysis - title TERPS is a mislabel to correct. Est. $20M point (range $15-40M, Medium confidence). Capture verdict: PURSUE - Flagship.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Pipeline: correct OPP-008 title to VA VIPPS (Phase II) — the flagship
Solicitation 36C10B26Q0107 is VA VIPPS (Phase II), not "TERPS" — the row
had carried the wrong name since intake. Rename OPP-008 and rewrite the
notes to the actual VIPPS scope (VistA/iFAMS/FORCE integration + AI/ML +
FedRAMP Mod + RMF; Best Value Trade-Off, FFP; Phase I closed 5/4/26).

Value ($20M) and stage unchanged, so no formula caches move; surgical XML
edit preserves all 252 caches. verify_parse.js: 11/11 pass, 0 drift.
</commit_message>
<xml_diff>
--- a/VBX_Command_Center_v1.xlsx
+++ b/VBX_Command_Center_v1.xlsx
@@ -18402,7 +18402,7 @@
       </c>
       <c r="B12" s="42" t="inlineStr">
         <is>
-          <t xml:space="preserve">VA TERPS Support (36C10B26Q0107)</t>
+          <t xml:space="preserve">VA VIPPS (Phase II) - VistA/iFAMS Integration (36C10B26Q0107)</t>
         </is>
       </c>
       <c r="C12" s="42" t="inlineStr">
@@ -18436,7 +18436,7 @@
       </c>
       <c r="J12" s="42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Teaming with The Enterprise Solutions (TES). Sol. 36C10B26Q0107 = VA VIPPS (Phase II) per capture analysis - title TERPS is a mislabel to correct. Est. $20M point (range $15-40M, Medium confidence). Capture verdict: PURSUE - Flagship.</t>
+          <t xml:space="preserve">Teaming with The Enterprise Solutions (TES). VA OIT; GSA MAS / SIN 54151S. Phase II only (Phase I closed 5/4/26). Best Value Trade-Off, FFP; PoP 12-mo base + 4 option yrs (close 7/1/2026). Scope: VistA / iFAMS / FORCE integration + AI/ML + FedRAMP Mod + RMF. Est. $20M point (range $15-40M; most likely $15-25M, Medium confidence). FLAGSHIP - PURSUE.</t>
         </is>
       </c>
     </row>

</xml_diff>